<commit_message>
test suites and common data provider
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/TestData.xlsx
+++ b/src/test/resources/excel/TestData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96e9be76c92faddd/Desktop/Framework_DDT/DDT_Framework_Jenkins/src/test/resources/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{6F016867-0A92-40A8-BF8A-0F988EC3D6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A88291C3-4964-4756-966E-877A3ABD1FBF}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{6F016867-0A92-40A8-BF8A-0F988EC3D6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0512801-55F8-4396-9439-81D485A482F4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{B171A020-8E69-434E-9B00-B5D99F73080C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B171A020-8E69-434E-9B00-B5D99F73080C}"/>
   </bookViews>
   <sheets>
-    <sheet name="TestCase002_AddCustomerTest" sheetId="1" r:id="rId1"/>
-    <sheet name="TestCase003_OpenAccountTest" sheetId="2" r:id="rId2"/>
+    <sheet name="Test_Suite" sheetId="3" r:id="rId1"/>
+    <sheet name="TestCase002_AddCustomerTest" sheetId="1" r:id="rId2"/>
+    <sheet name="TestCase003_OpenAccountTest" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
   <si>
     <t>FirstName</t>
   </si>
@@ -104,6 +105,33 @@
   </si>
   <si>
     <t>Account created successfully</t>
+  </si>
+  <si>
+    <t>Run Mode</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>TC_ID</t>
+  </si>
+  <si>
+    <t>RUN_MODE</t>
+  </si>
+  <si>
+    <t>TestCase001_BankManagerLogin</t>
+  </si>
+  <si>
+    <t>TestCase002_AddCustomerTest</t>
+  </si>
+  <si>
+    <t>TestCase003_OpenAccountTest</t>
+  </si>
+  <si>
+    <t>TestCase004_ShowCustomers</t>
   </si>
 </sst>
 </file>
@@ -119,12 +147,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -139,8 +173,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,69 +493,52 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CD089D2-2C2C-417D-8F85-AF9DBCD2DFB0}">
-  <dimension ref="A1:D4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8AD97E4-5CB3-435A-8AB0-82E8F0CA0DAB}">
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="4" max="4" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -529,8 +547,92 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CD089D2-2C2C-417D-8F85-AF9DBCD2DFB0}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5F7FD12-C7DD-4A87-B48B-96C7DC2F4A12}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" customWidth="1"/>
@@ -538,7 +640,7 @@
     <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -548,8 +650,11 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -559,8 +664,11 @@
       <c r="C2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -570,8 +678,11 @@
       <c r="C3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -580,6 +691,9 @@
       </c>
       <c r="C4" t="s">
         <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>